<commit_message>
视频工作流: 更新 等202个 — .gitignore, .gitignore, 523bd5f4b50b7c1c03ec6c1538a002aabc1935c0.data.json
</commit_message>
<xml_diff>
--- a/视频工作流/_proc/推进路线.xlsx
+++ b/视频工作流/_proc/推进路线.xlsx
@@ -11,7 +11,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="能力清单" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="判据阈值" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="批次计划" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="批次进度" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,9 +31,6 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -62,13 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -434,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -564,7 +559,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>turn</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -577,7 +572,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -607,7 +602,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>wave</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -620,7 +615,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -650,12 +645,12 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>run,brake</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>penetration_m,float_m,frame_jump_ratio</t>
+          <t>ground_penetration_m,contact_float_m,flight_apex_err,frame_jump_ratio</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -663,7 +658,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -693,12 +688,12 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>jump</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>float_m,penetration_m,energy_gain,frame_jump_ratio</t>
+          <t>contact_float_m,flight_apex_err,energy_gain,frame_jump_ratio</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -706,7 +701,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -736,12 +731,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>crouch,reach_grab</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>float_m,penetration_m,skate_cm_frame</t>
+          <t>float_m,penetration_m,skate_cm_frame,arm_reach</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -749,7 +744,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -779,7 +774,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>carry_prop</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -792,7 +787,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -822,7 +817,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>prop_release</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -835,7 +830,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -865,7 +860,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>rigid_body,toppling</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -878,7 +873,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -908,12 +903,12 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>stack</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>penetration_m,jitter_px</t>
+          <t>penetration_m</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
@@ -921,7 +916,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -951,7 +946,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>ramp</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -964,7 +959,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -994,7 +989,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>bounce</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1007,7 +1002,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1032,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>pendulum</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1050,7 +1045,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1075,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>rigid_body</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1093,7 +1088,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1118,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>kick,ball</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1136,7 +1131,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1166,7 +1161,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>throw,ball</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1179,7 +1174,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1209,7 +1204,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>catch,ball</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1222,7 +1217,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1247,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>push,box</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1265,7 +1260,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1290,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>rope</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1308,7 +1303,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1333,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>hinge_door</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1351,7 +1346,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1376,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>multi_actor,contact</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1394,7 +1389,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1419,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>multi_actor,throw,catch</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1437,7 +1432,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1462,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>multi_actor,quadruped</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1480,7 +1475,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1510,12 +1505,12 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>crowd_collide</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>penetration_m,jitter_px</t>
+          <t>penetration_m</t>
         </is>
       </c>
       <c r="H25" s="2" t="n">
@@ -1523,7 +1518,7 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1553,12 +1548,12 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>run,jump,reach_grab,roll</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>float_m,penetration_m,frame_jump_ratio</t>
+          <t>frame_jump_ratio,energy_gain</t>
         </is>
       </c>
       <c r="H26" s="2" t="n">
@@ -1566,7 +1561,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1596,7 +1591,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>carry_box</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -1609,7 +1604,7 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1634,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>throw,toppling</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -1652,7 +1647,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1677,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>climb</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -1695,7 +1690,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1725,12 +1720,12 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>stack,toppling</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>penetration_m,energy_gain</t>
+          <t>penetration_m,frame_jump_ratio</t>
         </is>
       </c>
       <c r="H30" s="2" t="n">
@@ -1738,7 +1733,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1763,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>run,ccd</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -1781,7 +1776,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1811,12 +1806,12 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>rigid_body,broadphase</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>penetration_m,energy_gain,jitter_px</t>
+          <t>penetration_m</t>
         </is>
       </c>
       <c r="H32" s="2" t="n">
@@ -1824,7 +1819,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1849,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>gravity_off</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -1867,7 +1862,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1897,7 +1892,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>friction</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -1910,7 +1905,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1940,12 +1935,12 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>overlap_resolve</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>penetration_m,jitter_px</t>
+          <t>penetration_m</t>
         </is>
       </c>
       <c r="H35" s="2" t="n">
@@ -1953,7 +1948,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>缺能力</t>
+          <t>PASS/FAIL待测</t>
         </is>
       </c>
     </row>
@@ -1995,6 +1990,178 @@
         <v>66</v>
       </c>
       <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>PASS/FAIL待测</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>G36</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>ADDITIVE 三能力接线：gaze/finger/page 叠加到 gait，下半身零污染</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>walk,gaze_shift,finger_tap,page_flip</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>lower_pollution,frame_jump_ratio</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>PASS/FAIL待测</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>G37</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>攀岩：三点支撑 / 支撑相零滑移 / 不穿壁</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>climb_rock</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>support_min,foot_slip_m,ground_penetration_m,frame_jump_ratio</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>PASS/FAIL待测</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>G38</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>鱼游：脊椎段长守恒 / Strouhal 区间 / 帧间平滑</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>fish_swim,fish_strouhal</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>seg_len_err,strouhal_lo,strouhal_hi,frame_jump_ratio</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>PASS/FAIL待测</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>G39</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>四足六步态：支撑足缺口 / 足端滑移 / 帧间平滑</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>quadruped</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>gait_contact_deficit,foot_slip_m,frame_jump_ratio</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
         <is>
           <t>PASS/FAIL待测</t>
         </is>
@@ -2011,7 +2178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2056,7 +2223,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -2081,7 +2248,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -2106,7 +2273,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -2131,7 +2298,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -2156,7 +2323,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -2181,7 +2348,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -2206,7 +2373,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -2231,7 +2398,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -2256,7 +2423,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -2281,7 +2448,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -2306,7 +2473,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -2331,7 +2498,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -2356,7 +2523,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -2381,7 +2548,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -2406,7 +2573,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -2431,7 +2598,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -2456,7 +2623,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -2481,7 +2648,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -2506,7 +2673,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -2531,7 +2698,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -2556,7 +2723,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -2581,7 +2748,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -2606,7 +2773,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -2614,7 +2781,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>D23</t>
+          <t>D23,G39</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -2631,7 +2798,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2656,7 +2823,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2681,7 +2848,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2706,7 +2873,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2731,7 +2898,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2756,7 +2923,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2781,7 +2948,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2806,7 +2973,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2831,7 +2998,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2856,7 +3023,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2879,7 +3046,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2897,12 +3064,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>prop_release</t>
+          <t>climb_rock</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>已有</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2912,7 +3079,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>B9</t>
+          <t>G37</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr"/>
@@ -2920,25 +3087,163 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
+          <t>finger_tap</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>已有</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>G36</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>fish_strouhal</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>已有</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>G38</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>fish_swim</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>已有</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>G38</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>gaze_shift</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>已有</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>G36</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>page_flip</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>已有</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>G36</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>prop_release</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>已有</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>B9</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
           <t>walk</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>已有</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>A1,F35</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr"/>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>A1,F35,G36</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2951,7 +3256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2985,11 +3290,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>skate_cm_frame</t>
+          <t>lower_pollution</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1</v>
+        <v>1e-09</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -2998,18 +3303,18 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Zhang et al.2018 foot skating s=v(2-2h/H), H=2.5cm; 动捕真值0.10cm/frame</t>
+          <t>UE Layered Blend per Bone: additive 只作用于 mask 覆盖骨，下半身零污染</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>float_m</t>
+          <t>box_rest_m</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0.05</v>
+        <v>1e-09</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -3018,38 +3323,38 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>ReinDiffuse(arXiv:2410.07296) Floating: 距地面最低关节&gt;5cm</t>
+          <t>放箱 detach 后 owner=world，箱体底面贴合台面（carry.box_release 契约）</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>feet_clip_m</t>
+          <t>skate_cm_frame</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>0.05</v>
+        <v>1</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>&gt;</t>
+          <t>&lt;</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>ReinDiffuse Clip: 双脚距离&lt;5cm</t>
+          <t>Zhang et al.2018 foot skating s=v(2-2h/H), H=2.5cm; 动捕真值0.10cm/frame</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>penetration_m</t>
+          <t>float_m</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -3058,38 +3363,38 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>SIGGRAPH Asia2025 Penetration Estimation(GJK+EPA); Box2D linear slop=0.01</t>
+          <t>ReinDiffuse(arXiv:2410.07296, Han et al.) §Evaluation Metrics 原文: 'Ground floating measures the distance between the ground and the lowest joint positions above the ground (&gt; 5 cm)' —— 5cm 阈值出自该文正文，非自定</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>jitter_px</t>
+          <t>feet_clip_m</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>&lt;</t>
+          <t>&gt;</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>SMPTE 视频质量评估：Jitter Score &lt;0.1px（高分辨率显示）</t>
+          <t>ReinDiffuse(arXiv:2410.07296) §Evaluation Metrics 原文: 'Foot clipping measures the distance between the left and right feet when it is less than a certain distance threshold (5 cm)' —— 5cm 阈值出自该文正文</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>frame_jump_ratio</t>
+          <t>penetration_m</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>3</v>
+        <v>0.005</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -3098,18 +3403,18 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>帧间位移/段内中位位移，比值过大即时间跳变</t>
+          <t>穿模深度：Box2D 官方 b2_linearSlop=0.005m (v2.4.1 b2_common.h:65)；实测 C16 max=5.57e-4</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>restitution_err</t>
+          <t>jitter_px</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -3118,18 +3423,18 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>COR: e=sqrt(h1/h0), h_n=h_0*e^(2n)（UA PH125 实验手册）</t>
+          <t>工程经验值(非SMPTE)：帧图灰度平均帧间绝对差；阈值由本工程自测标定</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>momentum_err</t>
+          <t>seg_penetration_m</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>0.02</v>
+        <v>0.005</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -3138,38 +3443,38 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>动量守恒 m1v1+m2v2 前后不变</t>
+          <t>骨段(胶囊)与球最短距离 &lt; 半径即穿模；容差同 Box2D 官方 slop=0.005m</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>energy_gain</t>
+          <t>frame_jump_ratio</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>&lt;=</t>
+          <t>&lt;</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>物理不守恒：总能量不得增加</t>
+          <t>帧间位移/段内中位位移，比值过大即时间跳变</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>arm_reach</t>
+          <t>pos_drift_m</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0.377</v>
+        <v>1e-06</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
@@ -3178,27 +3483,926 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Table M: ARM17.3+FOREARM15.5+WRIST-TO-GRIP3.8=36.6%H; Dempster 0.1877+0.151+0.038=0.3767H</t>
+          <t>动机出处：WorldCycle/CycleBench（港科大·武大·腾讯视频AI技术中心, 2026-08）RCS=重复循环稳定性，长程档381帧。阈值非取自该文，为本工程自测标定：双精度1440帧累加9.7e-13留6量级余量，单精度1.7e-4会FAIL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>mileage_rel_err</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>1e-09</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>GROMACS 辛积分：误差有界振荡不漂移；双精度实测2.9e-14留5量级余量，单精度5e-6会FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>peak_rate_dps</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>460</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>【自测标定值，非取自文献】动机出处 Zago et al., ISBS 2015 Proceedings 33(1):1335-1338，但该文样本为 10 名 U-13 亚精英球员/29 次试验/5m 运球后脚底半转身，人群与任务均与原地转身错配；且公开渠道未能核实原文报告过 '414 (90) °/s' 骨盆峰值角速度，故不引用该数值。460 °/s 系本工程自测标定：实测转身峰值 399.6 °/s（裕度 13%）；定标顺序为 1020→460 收紧方向，非放宽（见 A1 铁律：阈值先定标再跑测试）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>restitution_err</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>COR: e=sqrt(h1/h0), h_n=h_0*e^(2n)（UA PH125 实验手册）</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>momentum_err</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>动量守恒 m1v1+m2v2 前后不变</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>energy_gain</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>1e-09</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>物理不守恒：总能量不得增加(浮点容差 1e-9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>arm_reach</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>0.377</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Table M: ARM17.3+FOREARM15.5+WRIST-TO-GRIP3.8=36.6%H; Dempster 0.1877+0.151+0.038=0.3767H</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>elbow_reflex</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B18" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>&lt;=</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>肘ROM 过伸5°~屈145°(Neumann/Kinesiology, Musculoskeletal Key)；实测=反折帧计数</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>contact_float_m</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>接触相浮空：同 Box2D 官方 b2_linearSlop=0.005m (v2.4.1 b2_common.h:65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>ground_penetration_m</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>穿地深度：同 Box2D 官方 b2_linearSlop=0.005m (v2.4.1 b2_common.h:65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>flight_apex_err</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>抛体 Δs=g·T_F²/8(UA PH125 实验手册 Projectile Motion)，相对误差5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>flight_g_err</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>抛体轨迹二次拟合 a=-g/2(UA PH125 Projectile Motion 手册, 匀加速运动 y=y0+v0t-gt²/2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>silhouette_gap_px</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>2D Hausdorff between silhouette masks: sensitive to holes and missing limbs(Integrated Platform for Live 3D Human Reconstruction)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>silhouette_span_ratio</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>同上：剪影须覆盖头到脚，比值过小即缺肢体</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>mask_iou</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>IoU/Jaccard index（Jaccard P. 1912, New Phytologist 11:37-50, §相似度系数）；阈值 0.75 为本工程自测标定（实测 D22 剪影 IoU=0.9357 留 25% 余量）。撤除说明：原引 ResiHMR(arXiv:2604.28025) 主题为残肢人群单图 3D 人体网格恢复，与本判据无方法论关联，属语义贴牌，已撤除</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>foot_slip_m</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Foot skating/sliding artifact：支撑相足端世界位移（业界 foot sliding metric）；阈值本工程自测标定</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>strouhal_lo</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Triantafyllou 1993：生物巡航 St 0.2~0.4（下界）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>strouhal_hi</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>同上上界</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>seg_len_err</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Jakobsen 2001 Advanced Character Physics 距离约束：段长误差应收敛到 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>support_min</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>攀岩三点支撑（three points of contact）：任一时刻 ≥3 效应器固定</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>gait_contact_deficit</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Hildebrand 1965 四足步态分类：walk/crawl 全程有支撑、trot/pace 对角 2 足、bound/gallop 存在腾空相(期望 0)；实测不得低于期望</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>zmp_out_pct</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>ZMP 稳定性：ZMP 全序列落在支撑多边形（BoS）内则越界率 0；出处 HUMOS(arXiv:2409.03944) Dyn.Stability / BoSDist</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>bos_dist_m</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>同上：ZMP 到支撑多边形边界的最小距离（米），&lt;0 表示越界</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>jitter_accel</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Karunratanakul 2023 Jitter：关节加速度变化量均值，非像素级抖动；过大会表现为高频抽搐</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>pene_bone_m</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>PeneBone(业界骨级自穿透指标)：每骨以 2cm 为半径做胶囊，非相邻骨间最深穿透深度；2r=0.04 即半径和的几何上界</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>contact_f1</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>CHOIS 接触指标：预测接触与真值接触的 precision/recall/F1；此处真值取动作自身声明的支撑相</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>duty_factor_err</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Hildebrand 1965 三变量之一：占空比(触地时长/周期)，walk 类应 &gt;0.5；本项测实测与步态表期望值之差</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>phase_err</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>同上：相对相位(以 LH 为参考的触地滞后)，trot 对角同相 0.0/0.5；本项测实测与期望之差</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>wave_len_ratio</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>鱼类行波：体波波长/体长；鲹科巡航约 1 个体长量级，低于 0.5 说明行波未成形（出处 Triantafyllou 1993）</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>nan_count</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>IEEE 754：NaN 参与任何算术均传播为 NaN，一旦出现即静默污染整条轨迹。混合场景里 NaN 的典型成因是子系统坐标口径不一致（如 2D 足端未补 z）或除零；阈值 0 表示零容忍</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>xbody_penetration_m</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>跨实体穿模：与项目其余穿模判据同用 Box2D 官方 b2_linearSlop=0.005f(v2.4.1 b2_common.h:65)。不同实体的骨架定义不同，故用逐帧包围球（半径=该帧点集到质心的最大距离）比较，不逐骨段互比</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>min_arc_m</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>防「实体没接上时间轴」：总弧长而非首尾距离——圆周/往复运动首尾距离可为 0，用首尾距会把原地摆动误判成静止。3 秒 72 帧下完全静止为 0，0.01m 足以区分静止与真实微幅运动（绳末端 Verlet 收敛后残余摆动）</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>time_span_err_s</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>0.04166666666666666</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>时间轴同步：各实体覆盖时长之差不得超过一帧(24fps=0.0417s)。超过一帧即出现某些实体先结束/后开始的错位，与多轨合成的帧对齐要求一致</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>leaf_v_term_mps</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>树叶飘落终端速度上限取 0.5·√(2gh)（h=2m）：flutter 的终端速度必须显著低于同高度自由落体，否则说明阻力未起作用。实测 flutter 0.1645 m/s、tumbling 0.5533 m/s(出处 Wang &amp; Pesavento 2004 PRL; Andersen et al. 2005 JFM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>frac_max_disp_m</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>碎块飞散位移上限：超限说明断裂释放的能量数值爆炸（PBD bond 失效瞬间位置投影过冲）。实测 0.4961 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>water_spread_ratio</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>水柱冲击地面后横向铺展比（终态横向范围/初始横向范围）。小于 1 说明流体被约束成柱子、密度约束未求解，等于 1 说明粒子没动（出处 PBF Macklin &amp; Müller 2013）</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>water_rho_rel</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>PBF 不可压缩：静息后平均 |ρ/ρ0-1|。密度约束求解达标即应收敛到静息密度附近，实测 0.0145（1.45%）</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>cradle_th_mid_win_rad</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>牛顿摆中间球在首次碰撞后 0.25s 窗口内的最大角位移，取 0.05·θ0(θ0=0.60rad)。等质量弹性碰撞⇒速度交换、中间球保持静止，这是牛顿摆的可观测签名（出处 GAUGE arXiv:2608.05948）</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>cradle_th_last_win_rad</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>同窗口内末球最大角位移，取 0.5·θ0：末球应被弹到接近首球初始摆角</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>turntable_r_end_m</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>转台物块最终半径需大于初始半径 r0=0.10：离心力 mω²r 超过静摩擦锥μs·m·g 后必然向外滑移（ω=8rad/s 时 mω²r=6.4N &gt; μs·m·g=3.43N）</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>turntable_lateral_m</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>科氏力 -2mω×v_rel 产生横向偏转，区别于纯径向离心：无科氏项时横向位移恒为 0，故 1e-6 足以自证该项已生效</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>leaf_drift_m</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>flutter 必须有水平漂移：纯竖直下落说明升力项未起作用。实测 3.54 m（2m 落差下的滑翔）</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>leaf_swings</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>flutter 的定义是左右摆动滑翔（swing≥2 次），区别于直线下坠（出处 Andersen et al. 2005 JFM 双稳态分类）</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>frac_n_broken</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>墙被撞后必须有 bond 超过 strain_limit 而失效，否则等于没裂</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>frac_n_frag</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>裂开的定义是连通分量 &gt;1（出现独立碎块）；等于 1 说明只是整体位移</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>water_n_alive</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="C56" s="2">
+        <f>=</f>
+        <v/>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>PBF 粒子数守恒：出现 NaN 或逃逸流体即丢失质量。注意判有限须逐粒子取 axis=1，漏 axis 会退化成标量而恒过</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>cradle_energy_err</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>牛顿摆能量守恒：e=0.999 允许少量耗散，实测 0.0241。单摆积分用 dt=1/4000 保证摆本身不引入显著漂移</t>
         </is>
       </c>
     </row>
@@ -3511,445 +4715,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>用例</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>状态</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>判据实测</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>本轮结论</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>A1 直线行走</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>skate 0.6972cm/帧; float 0.02418m; feet_clip 0.1873m</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>修地面标定后转 PASS：gait 归一化坐标地面不在 0，必须先标定 GROUND_V</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>F35 超长视频</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>同 A1 采样</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>当前仅复用 A1 一周期，未真正测 1 分钟累积漂移，待补</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>A4 转身180</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>frame_jump 1.343; jitter 0.0592px</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>头滞后 &gt; 躯干滞后已验证；转身耗时 0.6s</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>A5 挥手</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>frame_jump 1.639</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>摆动/抬起幅度均腕&gt;肘&gt;肩，肘同向无反折</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>合计</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>PASS 4 / FAIL 0 / READY 2 / STUB 29 / ERROR 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>A3 原地跳跃</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>float 0m; frame_jump 2.415; energy_gain 1.47e-16</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>腾空段解析抛物线，蹬伸末速=起跳速、落地末速=0；弃用位移倍率判据(速度过零必虚高)，改加速度有界</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>A7 下蹲捡物</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>float 0m; arm_reach 0.3334m(&lt;0.377)</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>蹲到底时肩-物距 0.3334 在臂展内；判据应取接触时刻而非全程 max(初始站立肩高达 0.686 必 FAIL)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>判据修正</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>已改</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>energy_gain 阈值 0.0 → 1e-9</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>浮点残差 1.47e-16 被判不守恒，属判据过严非代码错；加浮点容差并注明出处</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>合计</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>PASS 6 / FAIL 0 / READY 2 / STUB 27 / ERROR 0</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="n"/>
-      <c r="D10" s="2" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>批次4</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>B8 拿杯子 / B9 放下杯子</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>PASS 10 / FAIL 0 / STUB 25</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>手心到杯心=杯半径+腕到抓握点；detach 无跳变(1.581)；穿透台面 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>批次5</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>C18 弹球 / C20 两球对撞</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>PASS 12 / FAIL 0 / STUB 23 / ERROR 0</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>新建 motion/rigid.py：Verlet 定步长积分 + 冲量法碰撞；COR 表 7 种材质</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>C18 弹球</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>restitution 2.19e-15; energy_gain -0.916; penetration 0</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>峰值离地 0.675→0.3797→0.2136→0.1201，严格 h·e^(2n)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>C20 两球对撞</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>momentum_err 0; penetration 0.0075m</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>等质量速度交换 (-1,2)；异质量末速 (0.3333, 4.3333) 动量守恒</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>修坑</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>积分器</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>半隐式欧拉 → Velocity Verlet</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>欧拉每步偏低 0.5·g·dt²，累积 0.048~0.062m 超阈值；Verlet 对常加速度精确</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>修坑</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>穿透修正</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>vc²=v1²-2g·pen</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>原符号反了导致反弹越弹越高</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>修坑</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>EXEC 契约</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>返回 (checks, extra) 元组</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>我返回了 dict，main 解包报 too many values to unpack</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>修坑</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>to_mp4 路径</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>motion.run 非 motion.character.render</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>按实际定义位置导入</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>D22</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>gap=0; span=1.035; iou=0.9357; pen=9.93e-16; mom=1.71e-14; 球心最低1.0846&gt;半径0.1114</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>第二人画在extra回调(掩膜后)，B10教训复用；判据分段量避免跨越虚高</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>待办</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>run_all.py 516行超纲(R2&gt;500)</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>需拆出A组/B8B9用例到 cases_base.py</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>motion包30条目&gt;R4上限20，待分组</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>